<commit_message>
Added data for Dec 2025
</commit_message>
<xml_diff>
--- a/data/FRS_cleaned/Dec/Fmn D Dec/Dec 2025-D.xlsx
+++ b/data/FRS_cleaned/Dec/Fmn D Dec/Dec 2025-D.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\fwDemo\data\FRS_cleaned\Dec\Fmn D Dec\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43681EDD-8024-4398-8852-37A23A1A79F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C22C1BE-F06F-4091-99FD-24BF5CF6E127}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A Vehicle" sheetId="10" r:id="rId1"/>
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1244" uniqueCount="769">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1247" uniqueCount="772">
   <si>
     <t>Ser</t>
   </si>
@@ -2678,13 +2678,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">  1 x VOR for eng assy demanded.
-01 x MUAs Cut of Relay Eng Generator 
-  2 x EOA for want of spares from H1/ F1. 
-   2 x EOA due to DRWO fwd to W1 / W2 ABW.
-01 x  Under MR at 33 CZW</t>
-  </si>
-  <si>
     <t>10 Armd Regt</t>
   </si>
   <si>
@@ -2711,6 +2704,23 @@
 01 x EOA for want of spares from H1/ F1
 01 x Defect Report raised, investigation carried out wef 3-11 Nov 25 in unit loc by team ex GCF Jabalpur. 
 01 x VOR for eng assy dmd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  1 x VOR for eng assy demanded.
+01 x MUAs Cut of Relay Eng Generator 
+   2 x EOA due to DRWO fwd to W1 / W2 ABW.
+01 x  Under MR at 33 CZW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+  2 x EOA for want of spares from H1/ F1. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+  1 x EOA for want of spares from H1/ F1. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 x VOR for eng assy demanded. </t>
   </si>
 </sst>
 </file>
@@ -3969,171 +3979,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -4146,6 +3991,171 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="3" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5126,80 +5136,80 @@
       <c r="U2" s="92"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" s="277" t="s">
+      <c r="A3" s="282" t="s">
         <v>43</v>
       </c>
-      <c r="B3" s="277"/>
-      <c r="C3" s="277"/>
-      <c r="D3" s="277"/>
-      <c r="E3" s="277"/>
-      <c r="F3" s="277"/>
-      <c r="G3" s="277"/>
-      <c r="H3" s="277"/>
-      <c r="I3" s="277"/>
-      <c r="J3" s="277"/>
-      <c r="K3" s="277"/>
-      <c r="L3" s="277"/>
-      <c r="M3" s="277"/>
-      <c r="N3" s="277"/>
-      <c r="O3" s="277"/>
-      <c r="P3" s="277"/>
-      <c r="Q3" s="277"/>
-      <c r="R3" s="277"/>
-      <c r="S3" s="277"/>
-      <c r="T3" s="277"/>
-      <c r="U3" s="277"/>
+      <c r="B3" s="282"/>
+      <c r="C3" s="282"/>
+      <c r="D3" s="282"/>
+      <c r="E3" s="282"/>
+      <c r="F3" s="282"/>
+      <c r="G3" s="282"/>
+      <c r="H3" s="282"/>
+      <c r="I3" s="282"/>
+      <c r="J3" s="282"/>
+      <c r="K3" s="282"/>
+      <c r="L3" s="282"/>
+      <c r="M3" s="282"/>
+      <c r="N3" s="282"/>
+      <c r="O3" s="282"/>
+      <c r="P3" s="282"/>
+      <c r="Q3" s="282"/>
+      <c r="R3" s="282"/>
+      <c r="S3" s="282"/>
+      <c r="T3" s="282"/>
+      <c r="U3" s="282"/>
     </row>
     <row r="4" spans="1:21" s="94" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="278" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="272" t="s">
+      <c r="A4" s="283" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="280" t="s">
         <v>17</v>
       </c>
       <c r="C4" s="93"/>
-      <c r="D4" s="278" t="s">
+      <c r="D4" s="283" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="278"/>
-      <c r="F4" s="278" t="s">
+      <c r="E4" s="283"/>
+      <c r="F4" s="283" t="s">
         <v>3</v>
       </c>
-      <c r="G4" s="278"/>
-      <c r="H4" s="278"/>
-      <c r="I4" s="278"/>
-      <c r="J4" s="278"/>
-      <c r="K4" s="278"/>
-      <c r="L4" s="278"/>
-      <c r="M4" s="278"/>
-      <c r="N4" s="272" t="s">
+      <c r="G4" s="283"/>
+      <c r="H4" s="283"/>
+      <c r="I4" s="283"/>
+      <c r="J4" s="283"/>
+      <c r="K4" s="283"/>
+      <c r="L4" s="283"/>
+      <c r="M4" s="283"/>
+      <c r="N4" s="280" t="s">
         <v>4</v>
       </c>
-      <c r="O4" s="272" t="s">
+      <c r="O4" s="280" t="s">
         <v>18</v>
       </c>
-      <c r="P4" s="278" t="s">
+      <c r="P4" s="283" t="s">
         <v>40</v>
       </c>
-      <c r="Q4" s="272" t="s">
+      <c r="Q4" s="280" t="s">
         <v>5</v>
       </c>
-      <c r="R4" s="272" t="s">
+      <c r="R4" s="280" t="s">
         <v>6</v>
       </c>
-      <c r="S4" s="272" t="s">
+      <c r="S4" s="280" t="s">
         <v>7</v>
       </c>
-      <c r="T4" s="272" t="s">
+      <c r="T4" s="280" t="s">
         <v>8</v>
       </c>
-      <c r="U4" s="272" t="s">
+      <c r="U4" s="280" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="94" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="278"/>
-      <c r="B5" s="272"/>
+      <c r="A5" s="283"/>
+      <c r="B5" s="280"/>
       <c r="C5" s="93" t="s">
         <v>44</v>
       </c>
@@ -5233,14 +5243,14 @@
       <c r="M5" s="95" t="s">
         <v>14</v>
       </c>
-      <c r="N5" s="272"/>
-      <c r="O5" s="272"/>
-      <c r="P5" s="278"/>
-      <c r="Q5" s="272"/>
-      <c r="R5" s="272"/>
-      <c r="S5" s="272"/>
-      <c r="T5" s="272"/>
-      <c r="U5" s="272"/>
+      <c r="N5" s="280"/>
+      <c r="O5" s="280"/>
+      <c r="P5" s="283"/>
+      <c r="Q5" s="280"/>
+      <c r="R5" s="280"/>
+      <c r="S5" s="280"/>
+      <c r="T5" s="280"/>
+      <c r="U5" s="280"/>
     </row>
     <row r="6" spans="1:21" s="94" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="95" t="s">
@@ -5306,10 +5316,10 @@
       </c>
     </row>
     <row r="7" spans="1:21" s="94" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="273" t="s">
+      <c r="A7" s="281" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="273"/>
+      <c r="B7" s="281"/>
       <c r="C7" s="96"/>
       <c r="D7" s="95"/>
       <c r="E7" s="95"/>
@@ -5337,7 +5347,7 @@
       <c r="B8" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="C8" s="327" t="s">
+      <c r="C8" s="272" t="s">
         <v>50</v>
       </c>
       <c r="D8" s="10">
@@ -5399,17 +5409,17 @@
         <v>94.594594594594597</v>
       </c>
       <c r="U8" s="25" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="36">
         <v>2</v>
       </c>
-      <c r="B9" s="274" t="s">
+      <c r="B9" s="277" t="s">
         <v>148</v>
       </c>
-      <c r="C9" s="328" t="s">
+      <c r="C9" s="273" t="s">
         <v>50</v>
       </c>
       <c r="D9" s="10">
@@ -5443,11 +5453,11 @@
         <v>0</v>
       </c>
       <c r="N9" s="11">
-        <f t="shared" ref="N9:N28" si="0">F9+G9+I9+J9</f>
+        <f t="shared" ref="N9:N26" si="0">F9+G9+I9+J9</f>
         <v>0</v>
       </c>
       <c r="O9" s="11">
-        <f t="shared" ref="O9:O28" si="1">H9+K9</f>
+        <f t="shared" ref="O9:O26" si="1">H9+K9</f>
         <v>2</v>
       </c>
       <c r="P9" s="11">
@@ -5478,8 +5488,8 @@
       <c r="A10" s="36">
         <v>3</v>
       </c>
-      <c r="B10" s="275"/>
-      <c r="C10" s="328" t="s">
+      <c r="B10" s="279"/>
+      <c r="C10" s="273" t="s">
         <v>51</v>
       </c>
       <c r="D10" s="10">
@@ -5548,8 +5558,8 @@
       <c r="A11" s="36">
         <v>4</v>
       </c>
-      <c r="B11" s="276"/>
-      <c r="C11" s="328" t="s">
+      <c r="B11" s="278"/>
+      <c r="C11" s="273" t="s">
         <v>756</v>
       </c>
       <c r="D11" s="10">
@@ -5618,10 +5628,10 @@
       <c r="A12" s="37">
         <v>5</v>
       </c>
-      <c r="B12" s="274" t="s">
+      <c r="B12" s="277" t="s">
         <v>149</v>
       </c>
-      <c r="C12" s="328" t="s">
+      <c r="C12" s="273" t="s">
         <v>758</v>
       </c>
       <c r="D12" s="10">
@@ -5690,8 +5700,8 @@
       <c r="A13" s="36">
         <v>6</v>
       </c>
-      <c r="B13" s="275"/>
-      <c r="C13" s="328" t="s">
+      <c r="B13" s="279"/>
+      <c r="C13" s="273" t="s">
         <v>52</v>
       </c>
       <c r="D13" s="10">
@@ -5710,7 +5720,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="26">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J13" s="26">
         <v>0</v>
@@ -5726,7 +5736,7 @@
       </c>
       <c r="N13" s="11">
         <f>F13+G13+I13+J13</f>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O13" s="11">
         <f t="shared" si="1"/>
@@ -5734,11 +5744,11 @@
       </c>
       <c r="P13" s="11">
         <f t="shared" si="2"/>
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="Q13" s="24">
         <f t="shared" si="6"/>
-        <v>6.557377049180328</v>
+        <v>3.278688524590164</v>
       </c>
       <c r="R13" s="24">
         <f t="shared" si="3"/>
@@ -5746,22 +5756,22 @@
       </c>
       <c r="S13" s="24">
         <f t="shared" si="4"/>
-        <v>88.52459016393442</v>
+        <v>91.803278688524586</v>
       </c>
       <c r="T13" s="24">
         <f t="shared" si="5"/>
-        <v>93.442622950819668</v>
+        <v>96.721311475409834</v>
       </c>
       <c r="U13" s="30" t="s">
-        <v>760</v>
+        <v>768</v>
       </c>
     </row>
     <row r="14" spans="1:21" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="36">
         <v>7</v>
       </c>
-      <c r="B14" s="275"/>
-      <c r="C14" s="328" t="s">
+      <c r="B14" s="279"/>
+      <c r="C14" s="273" t="s">
         <v>50</v>
       </c>
       <c r="D14" s="10">
@@ -5819,9 +5829,9 @@
       <c r="A15" s="36">
         <v>8</v>
       </c>
-      <c r="B15" s="275"/>
-      <c r="C15" s="328" t="s">
-        <v>761</v>
+      <c r="B15" s="279"/>
+      <c r="C15" s="273" t="s">
+        <v>760</v>
       </c>
       <c r="D15" s="10">
         <v>1</v>
@@ -5836,7 +5846,7 @@
         <v>0</v>
       </c>
       <c r="H15" s="10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I15" s="10">
         <v>0</v>
@@ -5859,11 +5869,11 @@
       </c>
       <c r="O15" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P15" s="11">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="Q15" s="24"/>
       <c r="R15" s="24"/>
@@ -5878,8 +5888,8 @@
       <c r="A16" s="37">
         <v>9</v>
       </c>
-      <c r="B16" s="276"/>
-      <c r="C16" s="328" t="s">
+      <c r="B16" s="278"/>
+      <c r="C16" s="273" t="s">
         <v>53</v>
       </c>
       <c r="D16" s="12">
@@ -5946,10 +5956,10 @@
       <c r="A17" s="36">
         <v>10</v>
       </c>
-      <c r="B17" s="279" t="s">
+      <c r="B17" s="276" t="s">
         <v>150</v>
       </c>
-      <c r="C17" s="328" t="s">
+      <c r="C17" s="273" t="s">
         <v>54</v>
       </c>
       <c r="D17" s="12">
@@ -6009,15 +6019,15 @@
         <v>100</v>
       </c>
       <c r="U17" s="31" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="36">
         <v>11</v>
       </c>
-      <c r="B18" s="279"/>
-      <c r="C18" s="328" t="s">
+      <c r="B18" s="276"/>
+      <c r="C18" s="273" t="s">
         <v>50</v>
       </c>
       <c r="D18" s="12">
@@ -6080,12 +6090,12 @@
       </c>
       <c r="U18" s="31"/>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A19" s="37">
         <v>12</v>
       </c>
-      <c r="B19" s="279"/>
-      <c r="C19" s="328" t="s">
+      <c r="B19" s="276"/>
+      <c r="C19" s="273" t="s">
         <v>758</v>
       </c>
       <c r="D19" s="12">
@@ -6104,7 +6114,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="11">
         <v>0</v>
@@ -6120,7 +6130,7 @@
       </c>
       <c r="N19" s="11">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="11">
         <f t="shared" si="1"/>
@@ -6128,11 +6138,11 @@
       </c>
       <c r="P19" s="11">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q19" s="24">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R19" s="24">
         <f t="shared" si="8"/>
@@ -6140,32 +6150,34 @@
       </c>
       <c r="S19" s="24">
         <f t="shared" si="9"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="T19" s="24">
         <f t="shared" si="5"/>
-        <v>100</v>
-      </c>
-      <c r="U19" s="31"/>
+        <v>0</v>
+      </c>
+      <c r="U19" s="31" t="s">
+        <v>770</v>
+      </c>
     </row>
     <row r="20" spans="1:21" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="36">
         <v>13</v>
       </c>
-      <c r="B20" s="274" t="s">
+      <c r="B20" s="277" t="s">
         <v>151</v>
       </c>
-      <c r="C20" s="327" t="s">
+      <c r="C20" s="272" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="329">
-        <v>1</v>
-      </c>
-      <c r="E20" s="329">
+      <c r="D20" s="274">
+        <v>1</v>
+      </c>
+      <c r="E20" s="274">
         <v>1</v>
       </c>
       <c r="F20" s="11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="11">
         <v>0</v>
@@ -6189,7 +6201,8 @@
         <v>0</v>
       </c>
       <c r="N20" s="11">
-        <v>0</v>
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
       <c r="O20" s="11">
         <f t="shared" si="1"/>
@@ -6197,11 +6210,11 @@
       </c>
       <c r="P20" s="11">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q20" s="24">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R20" s="24">
         <f t="shared" si="8"/>
@@ -6209,26 +6222,28 @@
       </c>
       <c r="S20" s="24">
         <f t="shared" si="9"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="T20" s="24">
         <f t="shared" si="5"/>
-        <v>100</v>
-      </c>
-      <c r="U20" s="31"/>
+        <v>0</v>
+      </c>
+      <c r="U20" s="31" t="s">
+        <v>771</v>
+      </c>
     </row>
     <row r="21" spans="1:21" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="36">
         <v>14</v>
       </c>
-      <c r="B21" s="275"/>
-      <c r="C21" s="330" t="s">
+      <c r="B21" s="279"/>
+      <c r="C21" s="275" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="329">
+      <c r="D21" s="274">
         <v>3</v>
       </c>
-      <c r="E21" s="329">
+      <c r="E21" s="274">
         <v>2</v>
       </c>
       <c r="F21" s="11">
@@ -6284,15 +6299,15 @@
         <v>50</v>
       </c>
       <c r="U21" s="31" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="22" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="37">
         <v>15</v>
       </c>
-      <c r="B22" s="275"/>
-      <c r="C22" s="327" t="s">
+      <c r="B22" s="279"/>
+      <c r="C22" s="272" t="s">
         <v>55</v>
       </c>
       <c r="D22" s="4">
@@ -6354,21 +6369,21 @@
         <v>0</v>
       </c>
       <c r="U22" s="31" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="23" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="36">
         <v>16</v>
       </c>
-      <c r="B23" s="275"/>
-      <c r="C23" s="327" t="s">
-        <v>764</v>
-      </c>
-      <c r="D23" s="329">
+      <c r="B23" s="279"/>
+      <c r="C23" s="272" t="s">
+        <v>763</v>
+      </c>
+      <c r="D23" s="274">
         <v>2</v>
       </c>
-      <c r="E23" s="329">
+      <c r="E23" s="274">
         <v>2</v>
       </c>
       <c r="F23" s="11">
@@ -6429,12 +6444,12 @@
       <c r="A24" s="36">
         <v>17</v>
       </c>
-      <c r="B24" s="276"/>
+      <c r="B24" s="278"/>
       <c r="C24" s="209" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="329"/>
-      <c r="E24" s="329">
+      <c r="D24" s="274"/>
+      <c r="E24" s="274">
         <v>1</v>
       </c>
       <c r="F24" s="11">
@@ -6490,17 +6505,17 @@
         <v>0</v>
       </c>
       <c r="U24" s="31" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="25" spans="1:21" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="36">
         <v>18</v>
       </c>
-      <c r="B25" s="274" t="s">
+      <c r="B25" s="277" t="s">
         <v>152</v>
       </c>
-      <c r="C25" s="328" t="s">
+      <c r="C25" s="273" t="s">
         <v>758</v>
       </c>
       <c r="D25" s="10">
@@ -6567,8 +6582,8 @@
       <c r="A26" s="37">
         <v>19</v>
       </c>
-      <c r="B26" s="276"/>
-      <c r="C26" s="328" t="s">
+      <c r="B26" s="278"/>
+      <c r="C26" s="273" t="s">
         <v>52</v>
       </c>
       <c r="D26" s="12">
@@ -6630,17 +6645,17 @@
         <v>87.5</v>
       </c>
       <c r="U26" s="27" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="27" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="36">
         <v>20</v>
       </c>
-      <c r="B27" s="274" t="s">
+      <c r="B27" s="277" t="s">
         <v>153</v>
       </c>
-      <c r="C27" s="328" t="s">
+      <c r="C27" s="273" t="s">
         <v>758</v>
       </c>
       <c r="D27" s="12">
@@ -6702,15 +6717,15 @@
         <v>75</v>
       </c>
       <c r="U27" s="25" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="28" spans="1:21" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="36">
         <v>21</v>
       </c>
-      <c r="B28" s="275"/>
-      <c r="C28" s="328" t="s">
+      <c r="B28" s="279"/>
+      <c r="C28" s="273" t="s">
         <v>52</v>
       </c>
       <c r="D28" s="12">
@@ -6772,14 +6787,14 @@
         <v>50</v>
       </c>
       <c r="U28" s="31" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
     </row>
     <row r="29" spans="1:21" ht="36" x14ac:dyDescent="0.25">
       <c r="A29" s="37">
         <v>22</v>
       </c>
-      <c r="B29" s="275"/>
+      <c r="B29" s="279"/>
       <c r="C29" s="98" t="s">
         <v>51</v>
       </c>
@@ -6814,31 +6829,31 @@
         <v>0</v>
       </c>
       <c r="N29" s="11">
-        <f t="shared" ref="N9:N30" si="10">F29+G29+I29+J29</f>
+        <f t="shared" ref="N29:N30" si="10">F29+G29+I29+J29</f>
         <v>1</v>
       </c>
       <c r="O29" s="11">
-        <f t="shared" ref="O9:O30" si="11">H29+K29</f>
+        <f t="shared" ref="O29:O30" si="11">H29+K29</f>
         <v>0</v>
       </c>
       <c r="P29" s="11">
-        <f t="shared" ref="P9:P30" si="12">E29-N29-O29</f>
+        <f t="shared" ref="P29:P30" si="12">E29-N29-O29</f>
         <v>1</v>
       </c>
       <c r="Q29" s="24">
-        <f t="shared" ref="Q16:Q30" si="13">N29/E29*100</f>
+        <f t="shared" ref="Q29:Q30" si="13">N29/E29*100</f>
         <v>50</v>
       </c>
       <c r="R29" s="24">
-        <f t="shared" ref="R16:R30" si="14">O29*100/E29</f>
+        <f t="shared" ref="R29:R30" si="14">O29*100/E29</f>
         <v>0</v>
       </c>
       <c r="S29" s="24">
-        <f t="shared" ref="S16:S30" si="15">P29*100/E29</f>
+        <f t="shared" ref="S29:S30" si="15">P29*100/E29</f>
         <v>50</v>
       </c>
       <c r="T29" s="24">
-        <f t="shared" ref="T9:T33" si="16">R29+S29</f>
+        <f t="shared" ref="T29:T33" si="16">R29+S29</f>
         <v>50</v>
       </c>
       <c r="U29" s="27" t="s">
@@ -6849,7 +6864,7 @@
       <c r="A30" s="36">
         <v>23</v>
       </c>
-      <c r="B30" s="276"/>
+      <c r="B30" s="278"/>
       <c r="C30" s="97" t="s">
         <v>50</v>
       </c>
@@ -6869,7 +6884,7 @@
         <v>0</v>
       </c>
       <c r="I30" s="11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J30" s="11">
         <v>0</v>
@@ -6885,7 +6900,7 @@
       </c>
       <c r="N30" s="11">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O30" s="11">
         <f t="shared" si="11"/>
@@ -6893,11 +6908,11 @@
       </c>
       <c r="P30" s="11">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q30" s="24">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="R30" s="24">
         <f t="shared" si="14"/>
@@ -6905,13 +6920,15 @@
       </c>
       <c r="S30" s="24">
         <f t="shared" si="15"/>
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="T30" s="24">
         <f t="shared" si="16"/>
-        <v>100</v>
-      </c>
-      <c r="U30" s="27"/>
+        <v>0</v>
+      </c>
+      <c r="U30" s="27" t="s">
+        <v>769</v>
+      </c>
     </row>
     <row r="31" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="36">
@@ -7083,12 +7100,6 @@
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="B17:B19"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="S4:S5"/>
-    <mergeCell ref="T4:T5"/>
-    <mergeCell ref="B20:B24"/>
     <mergeCell ref="U4:U5"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="B9:B11"/>
@@ -7103,6 +7114,12 @@
     <mergeCell ref="P4:P5"/>
     <mergeCell ref="Q4:Q5"/>
     <mergeCell ref="R4:R5"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="S4:S5"/>
+    <mergeCell ref="T4:T5"/>
+    <mergeCell ref="B20:B24"/>
   </mergeCells>
   <phoneticPr fontId="28" type="noConversion"/>
   <dataValidations count="3">
@@ -7150,44 +7167,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:38" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="280" t="s">
+      <c r="A1" s="287" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="281"/>
-      <c r="C1" s="281"/>
-      <c r="D1" s="281"/>
-      <c r="E1" s="281"/>
-      <c r="F1" s="281"/>
-      <c r="G1" s="281"/>
-      <c r="H1" s="281"/>
-      <c r="I1" s="281"/>
-      <c r="J1" s="281"/>
+      <c r="B1" s="288"/>
+      <c r="C1" s="288"/>
+      <c r="D1" s="288"/>
+      <c r="E1" s="288"/>
+      <c r="F1" s="288"/>
+      <c r="G1" s="288"/>
+      <c r="H1" s="288"/>
+      <c r="I1" s="288"/>
+      <c r="J1" s="288"/>
     </row>
     <row r="2" spans="1:38" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="281"/>
-      <c r="B2" s="281"/>
-      <c r="C2" s="281"/>
-      <c r="D2" s="281"/>
-      <c r="E2" s="281"/>
-      <c r="F2" s="281"/>
-      <c r="G2" s="281"/>
-      <c r="H2" s="281"/>
-      <c r="I2" s="281"/>
-      <c r="J2" s="281"/>
+      <c r="A2" s="288"/>
+      <c r="B2" s="288"/>
+      <c r="C2" s="288"/>
+      <c r="D2" s="288"/>
+      <c r="E2" s="288"/>
+      <c r="F2" s="288"/>
+      <c r="G2" s="288"/>
+      <c r="H2" s="288"/>
+      <c r="I2" s="288"/>
+      <c r="J2" s="288"/>
     </row>
     <row r="3" spans="1:38" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="281" t="s">
+      <c r="A3" s="288" t="s">
         <v>120</v>
       </c>
-      <c r="B3" s="281"/>
-      <c r="C3" s="281"/>
-      <c r="D3" s="281"/>
-      <c r="E3" s="281"/>
-      <c r="F3" s="281"/>
-      <c r="G3" s="281"/>
-      <c r="H3" s="281"/>
-      <c r="I3" s="281"/>
-      <c r="J3" s="281"/>
+      <c r="B3" s="288"/>
+      <c r="C3" s="288"/>
+      <c r="D3" s="288"/>
+      <c r="E3" s="288"/>
+      <c r="F3" s="288"/>
+      <c r="G3" s="288"/>
+      <c r="H3" s="288"/>
+      <c r="I3" s="288"/>
+      <c r="J3" s="288"/>
     </row>
     <row r="4" spans="1:38" s="122" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="119" t="s">
@@ -7196,14 +7213,14 @@
       <c r="B4" s="120" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="282" t="s">
+      <c r="C4" s="289" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="283"/>
-      <c r="E4" s="284"/>
-      <c r="F4" s="284"/>
-      <c r="G4" s="284"/>
-      <c r="H4" s="284"/>
+      <c r="D4" s="290"/>
+      <c r="E4" s="291"/>
+      <c r="F4" s="291"/>
+      <c r="G4" s="291"/>
+      <c r="H4" s="291"/>
       <c r="I4" s="121" t="s">
         <v>40</v>
       </c>
@@ -9684,10 +9701,10 @@
       <c r="J96" s="108"/>
     </row>
     <row r="97" spans="1:38" s="137" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="287" t="s">
+      <c r="A97" s="284" t="s">
         <v>75</v>
       </c>
-      <c r="B97" s="287"/>
+      <c r="B97" s="284"/>
       <c r="C97" s="169"/>
       <c r="D97" s="169"/>
       <c r="E97" s="169"/>
@@ -10728,6 +10745,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:J2"/>
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="A97:B97"/>
     <mergeCell ref="A100:B100"/>
     <mergeCell ref="A18:B18"/>
@@ -10735,11 +10757,6 @@
     <mergeCell ref="A71:B71"/>
     <mergeCell ref="A75:B75"/>
     <mergeCell ref="A78:B78"/>
-    <mergeCell ref="A1:J2"/>
-    <mergeCell ref="A3:J3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="A7:B7"/>
   </mergeCells>
   <phoneticPr fontId="28" type="noConversion"/>
   <conditionalFormatting sqref="A1">
@@ -10800,18 +10817,18 @@
       </c>
     </row>
     <row r="2" spans="1:27" ht="36.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="288" t="s">
+      <c r="A2" s="292" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="288"/>
-      <c r="C2" s="288"/>
-      <c r="D2" s="288"/>
-      <c r="E2" s="288"/>
-      <c r="F2" s="288"/>
-      <c r="G2" s="288"/>
-      <c r="H2" s="288"/>
-      <c r="I2" s="288"/>
-      <c r="J2" s="288"/>
+      <c r="B2" s="292"/>
+      <c r="C2" s="292"/>
+      <c r="D2" s="292"/>
+      <c r="E2" s="292"/>
+      <c r="F2" s="292"/>
+      <c r="G2" s="292"/>
+      <c r="H2" s="292"/>
+      <c r="I2" s="292"/>
+      <c r="J2" s="292"/>
     </row>
     <row r="3" spans="1:27" s="8" customFormat="1" ht="47.25" x14ac:dyDescent="0.2">
       <c r="A3" s="41" t="s">
@@ -10824,9 +10841,9 @@
         <v>2</v>
       </c>
       <c r="D3" s="42"/>
-      <c r="E3" s="289"/>
-      <c r="F3" s="289"/>
-      <c r="G3" s="289"/>
+      <c r="E3" s="293"/>
+      <c r="F3" s="293"/>
+      <c r="G3" s="293"/>
       <c r="H3" s="41" t="s">
         <v>4</v>
       </c>
@@ -10926,18 +10943,18 @@
       </c>
     </row>
     <row r="6" spans="1:27" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="290" t="s">
+      <c r="A6" s="294" t="s">
         <v>110</v>
       </c>
-      <c r="B6" s="291"/>
-      <c r="C6" s="291"/>
-      <c r="D6" s="291"/>
-      <c r="E6" s="291"/>
-      <c r="F6" s="291"/>
-      <c r="G6" s="291"/>
-      <c r="H6" s="291"/>
-      <c r="I6" s="291"/>
-      <c r="J6" s="292"/>
+      <c r="B6" s="295"/>
+      <c r="C6" s="295"/>
+      <c r="D6" s="295"/>
+      <c r="E6" s="295"/>
+      <c r="F6" s="295"/>
+      <c r="G6" s="295"/>
+      <c r="H6" s="295"/>
+      <c r="I6" s="295"/>
+      <c r="J6" s="296"/>
     </row>
     <row r="7" spans="1:27" ht="24" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="79" t="s">
@@ -16482,85 +16499,85 @@
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A2" s="293" t="s">
+      <c r="A2" s="297" t="s">
         <v>116</v>
       </c>
-      <c r="B2" s="293"/>
-      <c r="C2" s="293"/>
-      <c r="D2" s="293"/>
-      <c r="E2" s="293"/>
-      <c r="F2" s="293"/>
-      <c r="G2" s="293"/>
-      <c r="H2" s="293"/>
-      <c r="I2" s="293"/>
-      <c r="J2" s="293"/>
-      <c r="K2" s="293"/>
-      <c r="L2" s="293"/>
-      <c r="M2" s="293"/>
-      <c r="N2" s="293"/>
-      <c r="O2" s="293"/>
-      <c r="P2" s="293"/>
-      <c r="Q2" s="293"/>
-      <c r="R2" s="293"/>
-      <c r="S2" s="293"/>
-      <c r="T2" s="293"/>
+      <c r="B2" s="297"/>
+      <c r="C2" s="297"/>
+      <c r="D2" s="297"/>
+      <c r="E2" s="297"/>
+      <c r="F2" s="297"/>
+      <c r="G2" s="297"/>
+      <c r="H2" s="297"/>
+      <c r="I2" s="297"/>
+      <c r="J2" s="297"/>
+      <c r="K2" s="297"/>
+      <c r="L2" s="297"/>
+      <c r="M2" s="297"/>
+      <c r="N2" s="297"/>
+      <c r="O2" s="297"/>
+      <c r="P2" s="297"/>
+      <c r="Q2" s="297"/>
+      <c r="R2" s="297"/>
+      <c r="S2" s="297"/>
+      <c r="T2" s="297"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="117"/>
       <c r="B3" s="188"/>
-      <c r="R3" s="294"/>
-      <c r="S3" s="295"/>
-      <c r="T3" s="295"/>
+      <c r="R3" s="298"/>
+      <c r="S3" s="299"/>
+      <c r="T3" s="299"/>
     </row>
     <row r="4" spans="1:20" s="189" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="296" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="297" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="298" t="s">
+      <c r="A4" s="300" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="301" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="302" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="299"/>
-      <c r="E4" s="296" t="s">
+      <c r="D4" s="303"/>
+      <c r="E4" s="300" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="296"/>
-      <c r="G4" s="296"/>
-      <c r="H4" s="296"/>
-      <c r="I4" s="296"/>
-      <c r="J4" s="296"/>
-      <c r="K4" s="296"/>
-      <c r="L4" s="296"/>
-      <c r="M4" s="300" t="s">
+      <c r="F4" s="300"/>
+      <c r="G4" s="300"/>
+      <c r="H4" s="300"/>
+      <c r="I4" s="300"/>
+      <c r="J4" s="300"/>
+      <c r="K4" s="300"/>
+      <c r="L4" s="300"/>
+      <c r="M4" s="304" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="300" t="s">
+      <c r="N4" s="304" t="s">
         <v>18</v>
       </c>
-      <c r="O4" s="302" t="s">
+      <c r="O4" s="306" t="s">
         <v>40</v>
       </c>
-      <c r="P4" s="297" t="s">
+      <c r="P4" s="301" t="s">
         <v>5</v>
       </c>
-      <c r="Q4" s="297" t="s">
+      <c r="Q4" s="301" t="s">
         <v>6</v>
       </c>
-      <c r="R4" s="297" t="s">
+      <c r="R4" s="301" t="s">
         <v>7</v>
       </c>
-      <c r="S4" s="297" t="s">
+      <c r="S4" s="301" t="s">
         <v>8</v>
       </c>
-      <c r="T4" s="304" t="s">
+      <c r="T4" s="308" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:20" s="189" customFormat="1" ht="36" x14ac:dyDescent="0.25">
-      <c r="A5" s="296"/>
-      <c r="B5" s="297"/>
+      <c r="A5" s="300"/>
+      <c r="B5" s="301"/>
       <c r="C5" s="190" t="s">
         <v>10</v>
       </c>
@@ -16591,14 +16608,14 @@
       <c r="L5" s="191" t="s">
         <v>14</v>
       </c>
-      <c r="M5" s="301"/>
-      <c r="N5" s="301"/>
-      <c r="O5" s="303"/>
-      <c r="P5" s="297"/>
-      <c r="Q5" s="297"/>
-      <c r="R5" s="297"/>
-      <c r="S5" s="297"/>
-      <c r="T5" s="305"/>
+      <c r="M5" s="305"/>
+      <c r="N5" s="305"/>
+      <c r="O5" s="307"/>
+      <c r="P5" s="301"/>
+      <c r="Q5" s="301"/>
+      <c r="R5" s="301"/>
+      <c r="S5" s="301"/>
+      <c r="T5" s="309"/>
     </row>
     <row r="6" spans="1:20" s="189" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="191" t="s">
@@ -17948,72 +17965,72 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A2" s="308" t="s">
+      <c r="A2" s="312" t="s">
         <v>535</v>
       </c>
-      <c r="B2" s="308"/>
-      <c r="C2" s="308"/>
-      <c r="D2" s="308"/>
-      <c r="E2" s="308"/>
-      <c r="F2" s="308"/>
-      <c r="G2" s="308"/>
-      <c r="H2" s="308"/>
-      <c r="I2" s="308"/>
-      <c r="J2" s="308"/>
-      <c r="K2" s="308"/>
-      <c r="L2" s="308"/>
-      <c r="M2" s="308"/>
-      <c r="N2" s="308"/>
-      <c r="O2" s="308"/>
-      <c r="P2" s="308"/>
-      <c r="Q2" s="308"/>
+      <c r="B2" s="312"/>
+      <c r="C2" s="312"/>
+      <c r="D2" s="312"/>
+      <c r="E2" s="312"/>
+      <c r="F2" s="312"/>
+      <c r="G2" s="312"/>
+      <c r="H2" s="312"/>
+      <c r="I2" s="312"/>
+      <c r="J2" s="312"/>
+      <c r="K2" s="312"/>
+      <c r="L2" s="312"/>
+      <c r="M2" s="312"/>
+      <c r="N2" s="312"/>
+      <c r="O2" s="312"/>
+      <c r="P2" s="312"/>
+      <c r="Q2" s="312"/>
     </row>
     <row r="3" spans="1:17" s="199" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="309" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="306" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="311" t="s">
+      <c r="A3" s="313" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="310" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="315" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="311"/>
-      <c r="E3" s="311" t="s">
+      <c r="D3" s="315"/>
+      <c r="E3" s="315" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="311"/>
-      <c r="G3" s="311"/>
-      <c r="H3" s="311"/>
-      <c r="I3" s="311"/>
-      <c r="J3" s="306" t="s">
+      <c r="F3" s="315"/>
+      <c r="G3" s="315"/>
+      <c r="H3" s="315"/>
+      <c r="I3" s="315"/>
+      <c r="J3" s="310" t="s">
         <v>4</v>
       </c>
-      <c r="K3" s="306" t="s">
+      <c r="K3" s="310" t="s">
         <v>536</v>
       </c>
-      <c r="L3" s="306" t="s">
+      <c r="L3" s="310" t="s">
         <v>537</v>
       </c>
-      <c r="M3" s="306" t="s">
+      <c r="M3" s="310" t="s">
         <v>5</v>
       </c>
-      <c r="N3" s="306" t="s">
+      <c r="N3" s="310" t="s">
         <v>6</v>
       </c>
-      <c r="O3" s="306" t="s">
+      <c r="O3" s="310" t="s">
         <v>7</v>
       </c>
-      <c r="P3" s="306" t="s">
+      <c r="P3" s="310" t="s">
         <v>8</v>
       </c>
-      <c r="Q3" s="307" t="s">
+      <c r="Q3" s="311" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:17" s="204" customFormat="1" ht="105.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="310"/>
-      <c r="B4" s="306"/>
+      <c r="A4" s="314"/>
+      <c r="B4" s="310"/>
       <c r="C4" s="200" t="s">
         <v>10</v>
       </c>
@@ -18035,14 +18052,14 @@
       <c r="I4" s="202" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="306"/>
-      <c r="K4" s="306"/>
-      <c r="L4" s="306"/>
-      <c r="M4" s="306"/>
-      <c r="N4" s="306"/>
-      <c r="O4" s="306"/>
-      <c r="P4" s="306"/>
-      <c r="Q4" s="307"/>
+      <c r="J4" s="310"/>
+      <c r="K4" s="310"/>
+      <c r="L4" s="310"/>
+      <c r="M4" s="310"/>
+      <c r="N4" s="310"/>
+      <c r="O4" s="310"/>
+      <c r="P4" s="310"/>
+      <c r="Q4" s="311"/>
     </row>
     <row r="5" spans="1:17" s="209" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
@@ -21683,24 +21700,24 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="312" t="s">
+      <c r="A2" s="325" t="s">
         <v>627</v>
       </c>
-      <c r="B2" s="312"/>
-      <c r="C2" s="312"/>
-      <c r="D2" s="312"/>
-      <c r="E2" s="312"/>
-      <c r="F2" s="312"/>
-      <c r="G2" s="312"/>
-      <c r="H2" s="312"/>
-      <c r="I2" s="312"/>
-      <c r="J2" s="312"/>
-      <c r="K2" s="312"/>
-      <c r="L2" s="312"/>
-      <c r="M2" s="312"/>
-      <c r="N2" s="312"/>
-      <c r="O2" s="312"/>
-      <c r="P2" s="312"/>
+      <c r="B2" s="325"/>
+      <c r="C2" s="325"/>
+      <c r="D2" s="325"/>
+      <c r="E2" s="325"/>
+      <c r="F2" s="325"/>
+      <c r="G2" s="325"/>
+      <c r="H2" s="325"/>
+      <c r="I2" s="325"/>
+      <c r="J2" s="325"/>
+      <c r="K2" s="325"/>
+      <c r="L2" s="325"/>
+      <c r="M2" s="325"/>
+      <c r="N2" s="325"/>
+      <c r="O2" s="325"/>
+      <c r="P2" s="325"/>
     </row>
     <row r="3" spans="1:16" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A3" s="220" t="s">
@@ -21825,7 +21842,7 @@
       </c>
     </row>
     <row r="6" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="313">
+      <c r="A6" s="322">
         <v>1</v>
       </c>
       <c r="B6" s="238" t="s">
@@ -21847,7 +21864,7 @@
       <c r="P6" s="243"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="314"/>
+      <c r="A7" s="323"/>
       <c r="B7" s="237" t="s">
         <v>22</v>
       </c>
@@ -21898,7 +21915,7 @@
       <c r="P7" s="5"/>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="314"/>
+      <c r="A8" s="323"/>
       <c r="B8" s="237" t="s">
         <v>23</v>
       </c>
@@ -21950,7 +21967,7 @@
       <c r="P8" s="5"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="314"/>
+      <c r="A9" s="323"/>
       <c r="B9" s="237" t="s">
         <v>24</v>
       </c>
@@ -22002,7 +22019,7 @@
       <c r="P9" s="5"/>
     </row>
     <row r="10" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A10" s="314"/>
+      <c r="A10" s="323"/>
       <c r="B10" s="237" t="s">
         <v>25</v>
       </c>
@@ -22056,7 +22073,7 @@
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="315"/>
+      <c r="A11" s="324"/>
       <c r="B11" s="237" t="s">
         <v>26</v>
       </c>
@@ -22110,7 +22127,7 @@
       </c>
     </row>
     <row r="12" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="313">
+      <c r="A12" s="322">
         <v>2</v>
       </c>
       <c r="B12" s="238" t="s">
@@ -22158,7 +22175,7 @@
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="314"/>
+      <c r="A13" s="323"/>
       <c r="B13" s="237" t="s">
         <v>22</v>
       </c>
@@ -22212,7 +22229,7 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="314"/>
+      <c r="A14" s="323"/>
       <c r="B14" s="237" t="s">
         <v>23</v>
       </c>
@@ -22266,7 +22283,7 @@
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="315"/>
+      <c r="A15" s="324"/>
       <c r="B15" s="237" t="s">
         <v>24</v>
       </c>
@@ -22320,7 +22337,7 @@
       </c>
     </row>
     <row r="16" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="313">
+      <c r="A16" s="322">
         <v>3</v>
       </c>
       <c r="B16" s="238" t="s">
@@ -22368,7 +22385,7 @@
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="314"/>
+      <c r="A17" s="323"/>
       <c r="B17" s="237" t="s">
         <v>22</v>
       </c>
@@ -22422,7 +22439,7 @@
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="314"/>
+      <c r="A18" s="323"/>
       <c r="B18" s="237" t="s">
         <v>23</v>
       </c>
@@ -22476,7 +22493,7 @@
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A19" s="314"/>
+      <c r="A19" s="323"/>
       <c r="B19" s="237" t="s">
         <v>24</v>
       </c>
@@ -22530,7 +22547,7 @@
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A20" s="314"/>
+      <c r="A20" s="323"/>
       <c r="B20" s="237" t="s">
         <v>25</v>
       </c>
@@ -22584,7 +22601,7 @@
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A21" s="315"/>
+      <c r="A21" s="324"/>
       <c r="B21" s="237" t="s">
         <v>25</v>
       </c>
@@ -22638,7 +22655,7 @@
       </c>
     </row>
     <row r="22" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="313">
+      <c r="A22" s="322">
         <v>4</v>
       </c>
       <c r="B22" s="238" t="s">
@@ -22686,7 +22703,7 @@
       </c>
     </row>
     <row r="23" spans="1:16" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="314"/>
+      <c r="A23" s="323"/>
       <c r="B23" s="237" t="s">
         <v>22</v>
       </c>
@@ -22740,7 +22757,7 @@
       </c>
     </row>
     <row r="24" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="314"/>
+      <c r="A24" s="323"/>
       <c r="B24" s="237" t="s">
         <v>23</v>
       </c>
@@ -22794,7 +22811,7 @@
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A25" s="314"/>
+      <c r="A25" s="323"/>
       <c r="B25" s="237" t="s">
         <v>24</v>
       </c>
@@ -22848,7 +22865,7 @@
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A26" s="315"/>
+      <c r="A26" s="324"/>
       <c r="B26" s="237" t="s">
         <v>25</v>
       </c>
@@ -22902,7 +22919,7 @@
       </c>
     </row>
     <row r="27" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="313">
+      <c r="A27" s="322">
         <v>5</v>
       </c>
       <c r="B27" s="238" t="s">
@@ -22950,7 +22967,7 @@
       </c>
     </row>
     <row r="28" spans="1:16" ht="85.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="314"/>
+      <c r="A28" s="323"/>
       <c r="B28" s="237" t="s">
         <v>22</v>
       </c>
@@ -23004,7 +23021,7 @@
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A29" s="315"/>
+      <c r="A29" s="324"/>
       <c r="B29" s="237" t="s">
         <v>23</v>
       </c>
@@ -23058,7 +23075,7 @@
       </c>
     </row>
     <row r="30" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="313">
+      <c r="A30" s="322">
         <v>6</v>
       </c>
       <c r="B30" s="238" t="s">
@@ -23106,7 +23123,7 @@
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A31" s="314"/>
+      <c r="A31" s="323"/>
       <c r="B31" s="237" t="s">
         <v>22</v>
       </c>
@@ -23160,7 +23177,7 @@
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A32" s="314"/>
+      <c r="A32" s="323"/>
       <c r="B32" s="237" t="s">
         <v>23</v>
       </c>
@@ -23214,7 +23231,7 @@
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A33" s="314"/>
+      <c r="A33" s="323"/>
       <c r="B33" s="237" t="s">
         <v>24</v>
       </c>
@@ -23268,7 +23285,7 @@
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A34" s="314"/>
+      <c r="A34" s="323"/>
       <c r="B34" s="237" t="s">
         <v>25</v>
       </c>
@@ -23322,7 +23339,7 @@
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A35" s="315"/>
+      <c r="A35" s="324"/>
       <c r="B35" s="237" t="s">
         <v>26</v>
       </c>
@@ -23376,7 +23393,7 @@
       </c>
     </row>
     <row r="36" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A36" s="313">
+      <c r="A36" s="322">
         <v>7</v>
       </c>
       <c r="B36" s="238" t="s">
@@ -23424,7 +23441,7 @@
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A37" s="314"/>
+      <c r="A37" s="323"/>
       <c r="B37" s="237" t="s">
         <v>22</v>
       </c>
@@ -23478,7 +23495,7 @@
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A38" s="314"/>
+      <c r="A38" s="323"/>
       <c r="B38" s="237" t="s">
         <v>23</v>
       </c>
@@ -23532,7 +23549,7 @@
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A39" s="314"/>
+      <c r="A39" s="323"/>
       <c r="B39" s="237" t="s">
         <v>24</v>
       </c>
@@ -23586,7 +23603,7 @@
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A40" s="315"/>
+      <c r="A40" s="324"/>
       <c r="B40" s="237" t="s">
         <v>25</v>
       </c>
@@ -23640,7 +23657,7 @@
       </c>
     </row>
     <row r="41" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A41" s="313">
+      <c r="A41" s="322">
         <v>8</v>
       </c>
       <c r="B41" s="238" t="s">
@@ -23688,7 +23705,7 @@
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A42" s="314"/>
+      <c r="A42" s="323"/>
       <c r="B42" s="237" t="s">
         <v>22</v>
       </c>
@@ -23740,7 +23757,7 @@
       <c r="P42" s="5"/>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A43" s="315"/>
+      <c r="A43" s="324"/>
       <c r="B43" s="237" t="s">
         <v>23</v>
       </c>
@@ -23794,7 +23811,7 @@
       </c>
     </row>
     <row r="44" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A44" s="313">
+      <c r="A44" s="322">
         <v>9</v>
       </c>
       <c r="B44" s="238" t="s">
@@ -23842,7 +23859,7 @@
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A45" s="314"/>
+      <c r="A45" s="323"/>
       <c r="B45" s="237" t="s">
         <v>22</v>
       </c>
@@ -23896,7 +23913,7 @@
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A46" s="314"/>
+      <c r="A46" s="323"/>
       <c r="B46" s="237" t="s">
         <v>23</v>
       </c>
@@ -23950,7 +23967,7 @@
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A47" s="314"/>
+      <c r="A47" s="323"/>
       <c r="B47" s="237" t="s">
         <v>24</v>
       </c>
@@ -24004,7 +24021,7 @@
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A48" s="315"/>
+      <c r="A48" s="324"/>
       <c r="B48" s="237" t="s">
         <v>25</v>
       </c>
@@ -24058,7 +24075,7 @@
       </c>
     </row>
     <row r="49" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="313">
+      <c r="A49" s="322">
         <v>10</v>
       </c>
       <c r="B49" s="238" t="s">
@@ -24106,7 +24123,7 @@
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A50" s="314"/>
+      <c r="A50" s="323"/>
       <c r="B50" s="237" t="s">
         <v>22</v>
       </c>
@@ -24160,7 +24177,7 @@
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" s="314"/>
+      <c r="A51" s="323"/>
       <c r="B51" s="237" t="s">
         <v>23</v>
       </c>
@@ -24214,7 +24231,7 @@
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A52" s="314"/>
+      <c r="A52" s="323"/>
       <c r="B52" s="237" t="s">
         <v>24</v>
       </c>
@@ -24268,7 +24285,7 @@
       </c>
     </row>
     <row r="53" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A53" s="315"/>
+      <c r="A53" s="324"/>
       <c r="B53" s="237" t="s">
         <v>25</v>
       </c>
@@ -24322,7 +24339,7 @@
       </c>
     </row>
     <row r="54" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="313">
+      <c r="A54" s="322">
         <v>11</v>
       </c>
       <c r="B54" s="238" t="s">
@@ -24370,7 +24387,7 @@
       </c>
     </row>
     <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A55" s="314"/>
+      <c r="A55" s="323"/>
       <c r="B55" s="237" t="s">
         <v>22</v>
       </c>
@@ -24424,7 +24441,7 @@
       </c>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A56" s="315"/>
+      <c r="A56" s="324"/>
       <c r="B56" s="237" t="s">
         <v>23</v>
       </c>
@@ -24478,7 +24495,7 @@
       </c>
     </row>
     <row r="57" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A57" s="313">
+      <c r="A57" s="322">
         <v>12</v>
       </c>
       <c r="B57" s="238" t="s">
@@ -24526,7 +24543,7 @@
       </c>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A58" s="315"/>
+      <c r="A58" s="324"/>
       <c r="B58" s="237" t="s">
         <v>22</v>
       </c>
@@ -24580,7 +24597,7 @@
       </c>
     </row>
     <row r="59" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A59" s="313">
+      <c r="A59" s="322">
         <v>13</v>
       </c>
       <c r="B59" s="238" t="s">
@@ -24628,7 +24645,7 @@
       </c>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A60" s="314"/>
+      <c r="A60" s="323"/>
       <c r="B60" s="237" t="s">
         <v>22</v>
       </c>
@@ -24682,7 +24699,7 @@
       </c>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A61" s="315"/>
+      <c r="A61" s="324"/>
       <c r="B61" s="237" t="s">
         <v>23</v>
       </c>
@@ -24736,7 +24753,7 @@
       </c>
     </row>
     <row r="62" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A62" s="313">
+      <c r="A62" s="322">
         <v>14</v>
       </c>
       <c r="B62" s="238" t="s">
@@ -24784,7 +24801,7 @@
       </c>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A63" s="314"/>
+      <c r="A63" s="323"/>
       <c r="B63" s="237" t="s">
         <v>22</v>
       </c>
@@ -24838,7 +24855,7 @@
       </c>
     </row>
     <row r="64" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A64" s="315"/>
+      <c r="A64" s="324"/>
       <c r="B64" s="237" t="s">
         <v>23</v>
       </c>
@@ -24892,7 +24909,7 @@
       </c>
     </row>
     <row r="65" spans="1:16" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A65" s="313">
+      <c r="A65" s="322">
         <v>15</v>
       </c>
       <c r="B65" s="238" t="s">
@@ -24940,7 +24957,7 @@
       </c>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A66" s="314"/>
+      <c r="A66" s="323"/>
       <c r="B66" s="237" t="s">
         <v>22</v>
       </c>
@@ -24994,7 +25011,7 @@
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A67" s="315"/>
+      <c r="A67" s="324"/>
       <c r="B67" s="237" t="s">
         <v>23</v>
       </c>
@@ -25097,10 +25114,10 @@
       <c r="A69" s="23">
         <v>16</v>
       </c>
-      <c r="B69" s="316" t="s">
+      <c r="B69" s="318" t="s">
         <v>559</v>
       </c>
-      <c r="C69" s="317"/>
+      <c r="C69" s="319"/>
       <c r="D69" s="244">
         <v>32</v>
       </c>
@@ -25148,10 +25165,10 @@
       <c r="A70" s="23">
         <v>17</v>
       </c>
-      <c r="B70" s="316" t="s">
+      <c r="B70" s="318" t="s">
         <v>561</v>
       </c>
-      <c r="C70" s="317"/>
+      <c r="C70" s="319"/>
       <c r="D70" s="244">
         <v>388</v>
       </c>
@@ -25202,10 +25219,10 @@
       <c r="A71" s="23">
         <v>18</v>
       </c>
-      <c r="B71" s="316" t="s">
+      <c r="B71" s="318" t="s">
         <v>562</v>
       </c>
-      <c r="C71" s="317"/>
+      <c r="C71" s="319"/>
       <c r="D71" s="244">
         <v>215</v>
       </c>
@@ -25255,10 +25272,10 @@
       <c r="A72" s="23">
         <v>19</v>
       </c>
-      <c r="B72" s="316" t="s">
+      <c r="B72" s="318" t="s">
         <v>563</v>
       </c>
-      <c r="C72" s="317"/>
+      <c r="C72" s="319"/>
       <c r="D72" s="244">
         <v>24</v>
       </c>
@@ -25308,10 +25325,10 @@
       <c r="A73" s="23">
         <v>20</v>
       </c>
-      <c r="B73" s="316" t="s">
+      <c r="B73" s="318" t="s">
         <v>564</v>
       </c>
-      <c r="C73" s="317"/>
+      <c r="C73" s="319"/>
       <c r="D73" s="244">
         <v>130</v>
       </c>
@@ -25361,10 +25378,10 @@
       <c r="A74" s="23">
         <v>21</v>
       </c>
-      <c r="B74" s="316" t="s">
+      <c r="B74" s="318" t="s">
         <v>565</v>
       </c>
-      <c r="C74" s="317"/>
+      <c r="C74" s="319"/>
       <c r="D74" s="244">
         <v>106</v>
       </c>
@@ -25414,10 +25431,10 @@
       <c r="A75" s="255">
         <v>22</v>
       </c>
-      <c r="B75" s="316" t="s">
+      <c r="B75" s="318" t="s">
         <v>567</v>
       </c>
-      <c r="C75" s="317"/>
+      <c r="C75" s="319"/>
       <c r="D75" s="256">
         <v>8</v>
       </c>
@@ -25467,10 +25484,10 @@
       <c r="A76" s="260">
         <v>23</v>
       </c>
-      <c r="B76" s="316" t="s">
+      <c r="B76" s="318" t="s">
         <v>569</v>
       </c>
-      <c r="C76" s="317"/>
+      <c r="C76" s="319"/>
       <c r="D76" s="244">
         <v>5</v>
       </c>
@@ -25521,10 +25538,10 @@
       <c r="A77" s="23">
         <v>24</v>
       </c>
-      <c r="B77" s="316" t="s">
+      <c r="B77" s="318" t="s">
         <v>570</v>
       </c>
-      <c r="C77" s="317"/>
+      <c r="C77" s="319"/>
       <c r="D77" s="244">
         <v>14</v>
       </c>
@@ -25575,10 +25592,10 @@
       <c r="A78" s="23">
         <v>25</v>
       </c>
-      <c r="B78" s="316" t="s">
+      <c r="B78" s="318" t="s">
         <v>572</v>
       </c>
-      <c r="C78" s="317"/>
+      <c r="C78" s="319"/>
       <c r="D78" s="244">
         <v>0</v>
       </c>
@@ -25629,10 +25646,10 @@
       <c r="A79" s="260">
         <v>26</v>
       </c>
-      <c r="B79" s="316" t="s">
+      <c r="B79" s="318" t="s">
         <v>574</v>
       </c>
-      <c r="C79" s="317"/>
+      <c r="C79" s="319"/>
       <c r="D79" s="244">
         <v>0</v>
       </c>
@@ -25683,10 +25700,10 @@
       <c r="A80" s="23">
         <v>27</v>
       </c>
-      <c r="B80" s="316" t="s">
+      <c r="B80" s="318" t="s">
         <v>576</v>
       </c>
-      <c r="C80" s="317"/>
+      <c r="C80" s="319"/>
       <c r="D80" s="244">
         <v>161</v>
       </c>
@@ -25783,10 +25800,10 @@
       <c r="A82" s="23">
         <v>28</v>
       </c>
-      <c r="B82" s="318" t="s">
+      <c r="B82" s="320" t="s">
         <v>578</v>
       </c>
-      <c r="C82" s="319"/>
+      <c r="C82" s="321"/>
       <c r="D82" s="244">
         <v>304</v>
       </c>
@@ -25836,10 +25853,10 @@
       <c r="A83" s="260">
         <v>29</v>
       </c>
-      <c r="B83" s="318" t="s">
+      <c r="B83" s="320" t="s">
         <v>579</v>
       </c>
-      <c r="C83" s="319"/>
+      <c r="C83" s="321"/>
       <c r="D83" s="244">
         <v>16</v>
       </c>
@@ -25887,10 +25904,10 @@
       <c r="A84" s="260">
         <v>30</v>
       </c>
-      <c r="B84" s="318" t="s">
+      <c r="B84" s="320" t="s">
         <v>580</v>
       </c>
-      <c r="C84" s="319"/>
+      <c r="C84" s="321"/>
       <c r="D84" s="244">
         <v>27</v>
       </c>
@@ -25939,10 +25956,10 @@
       <c r="A85" s="261">
         <v>31</v>
       </c>
-      <c r="B85" s="318" t="s">
+      <c r="B85" s="320" t="s">
         <v>581</v>
       </c>
-      <c r="C85" s="319"/>
+      <c r="C85" s="321"/>
       <c r="D85" s="262">
         <v>52</v>
       </c>
@@ -25993,10 +26010,10 @@
       <c r="A86" s="260">
         <v>32</v>
       </c>
-      <c r="B86" s="318" t="s">
+      <c r="B86" s="320" t="s">
         <v>582</v>
       </c>
-      <c r="C86" s="319"/>
+      <c r="C86" s="321"/>
       <c r="D86" s="244">
         <v>47</v>
       </c>
@@ -26045,10 +26062,10 @@
       <c r="A87" s="260">
         <v>33</v>
       </c>
-      <c r="B87" s="318" t="s">
+      <c r="B87" s="320" t="s">
         <v>583</v>
       </c>
-      <c r="C87" s="319"/>
+      <c r="C87" s="321"/>
       <c r="D87" s="244">
         <v>0</v>
       </c>
@@ -26145,10 +26162,10 @@
       <c r="A89" s="260">
         <v>34</v>
       </c>
-      <c r="B89" s="316" t="s">
+      <c r="B89" s="318" t="s">
         <v>584</v>
       </c>
-      <c r="C89" s="317"/>
+      <c r="C89" s="319"/>
       <c r="D89" s="244">
         <v>411</v>
       </c>
@@ -26199,10 +26216,10 @@
       <c r="A90" s="266">
         <v>35</v>
       </c>
-      <c r="B90" s="316" t="s">
+      <c r="B90" s="318" t="s">
         <v>586</v>
       </c>
-      <c r="C90" s="317"/>
+      <c r="C90" s="319"/>
       <c r="D90" s="244">
         <v>188</v>
       </c>
@@ -26253,10 +26270,10 @@
       <c r="A91" s="23">
         <v>36</v>
       </c>
-      <c r="B91" s="316" t="s">
+      <c r="B91" s="318" t="s">
         <v>587</v>
       </c>
-      <c r="C91" s="317"/>
+      <c r="C91" s="319"/>
       <c r="D91" s="244">
         <v>677</v>
       </c>
@@ -26307,10 +26324,10 @@
       <c r="A92" s="267">
         <v>37</v>
       </c>
-      <c r="B92" s="316" t="s">
+      <c r="B92" s="318" t="s">
         <v>588</v>
       </c>
-      <c r="C92" s="317"/>
+      <c r="C92" s="319"/>
       <c r="D92" s="244">
         <v>1065</v>
       </c>
@@ -26360,10 +26377,10 @@
       <c r="A93" s="260">
         <v>38</v>
       </c>
-      <c r="B93" s="316" t="s">
+      <c r="B93" s="318" t="s">
         <v>589</v>
       </c>
-      <c r="C93" s="317"/>
+      <c r="C93" s="319"/>
       <c r="D93" s="244">
         <v>0</v>
       </c>
@@ -26412,10 +26429,10 @@
       <c r="A94" s="260">
         <v>39</v>
       </c>
-      <c r="B94" s="316" t="s">
+      <c r="B94" s="318" t="s">
         <v>590</v>
       </c>
-      <c r="C94" s="317"/>
+      <c r="C94" s="319"/>
       <c r="D94" s="244">
         <v>0</v>
       </c>
@@ -26466,10 +26483,10 @@
       <c r="A95" s="23">
         <v>40</v>
       </c>
-      <c r="B95" s="316" t="s">
+      <c r="B95" s="318" t="s">
         <v>592</v>
       </c>
-      <c r="C95" s="317"/>
+      <c r="C95" s="319"/>
       <c r="D95" s="244">
         <v>36</v>
       </c>
@@ -26520,10 +26537,10 @@
       <c r="A96" s="260">
         <v>41</v>
       </c>
-      <c r="B96" s="316" t="s">
+      <c r="B96" s="318" t="s">
         <v>594</v>
       </c>
-      <c r="C96" s="317"/>
+      <c r="C96" s="319"/>
       <c r="D96" s="244">
         <v>0</v>
       </c>
@@ -26574,10 +26591,10 @@
       <c r="A97" s="260">
         <v>42</v>
       </c>
-      <c r="B97" s="316" t="s">
+      <c r="B97" s="318" t="s">
         <v>596</v>
       </c>
-      <c r="C97" s="317"/>
+      <c r="C97" s="319"/>
       <c r="D97" s="244">
         <v>0</v>
       </c>
@@ -26628,10 +26645,10 @@
       <c r="A98" s="260">
         <v>43</v>
       </c>
-      <c r="B98" s="316" t="s">
+      <c r="B98" s="318" t="s">
         <v>597</v>
       </c>
-      <c r="C98" s="317"/>
+      <c r="C98" s="319"/>
       <c r="D98" s="244">
         <v>58</v>
       </c>
@@ -26682,10 +26699,10 @@
       <c r="A99" s="23">
         <v>44</v>
       </c>
-      <c r="B99" s="316" t="s">
+      <c r="B99" s="318" t="s">
         <v>598</v>
       </c>
-      <c r="C99" s="317"/>
+      <c r="C99" s="319"/>
       <c r="D99" s="244">
         <v>1968</v>
       </c>
@@ -26735,10 +26752,10 @@
       <c r="A100" s="260">
         <v>45</v>
       </c>
-      <c r="B100" s="316" t="s">
+      <c r="B100" s="318" t="s">
         <v>600</v>
       </c>
-      <c r="C100" s="317"/>
+      <c r="C100" s="319"/>
       <c r="D100" s="244">
         <v>171</v>
       </c>
@@ -26787,10 +26804,10 @@
       <c r="A101" s="260">
         <v>46</v>
       </c>
-      <c r="B101" s="316" t="s">
+      <c r="B101" s="318" t="s">
         <v>601</v>
       </c>
-      <c r="C101" s="317"/>
+      <c r="C101" s="319"/>
       <c r="D101" s="244">
         <v>0</v>
       </c>
@@ -26841,10 +26858,10 @@
       <c r="A102" s="260">
         <v>47</v>
       </c>
-      <c r="B102" s="316" t="s">
+      <c r="B102" s="318" t="s">
         <v>602</v>
       </c>
-      <c r="C102" s="317"/>
+      <c r="C102" s="319"/>
       <c r="D102" s="244">
         <v>36</v>
       </c>
@@ -26895,10 +26912,10 @@
       <c r="A103" s="260">
         <v>48</v>
       </c>
-      <c r="B103" s="316" t="s">
+      <c r="B103" s="318" t="s">
         <v>603</v>
       </c>
-      <c r="C103" s="317"/>
+      <c r="C103" s="319"/>
       <c r="D103" s="244">
         <v>175</v>
       </c>
@@ -26949,10 +26966,10 @@
       <c r="A104" s="260">
         <v>49</v>
       </c>
-      <c r="B104" s="316" t="s">
+      <c r="B104" s="318" t="s">
         <v>605</v>
       </c>
-      <c r="C104" s="317"/>
+      <c r="C104" s="319"/>
       <c r="D104" s="244">
         <v>8</v>
       </c>
@@ -27003,10 +27020,10 @@
       <c r="A105" s="260">
         <v>50</v>
       </c>
-      <c r="B105" s="316" t="s">
+      <c r="B105" s="318" t="s">
         <v>606</v>
       </c>
-      <c r="C105" s="317"/>
+      <c r="C105" s="319"/>
       <c r="D105" s="244">
         <v>440</v>
       </c>
@@ -27055,10 +27072,10 @@
       <c r="A106" s="260">
         <v>51</v>
       </c>
-      <c r="B106" s="316" t="s">
+      <c r="B106" s="318" t="s">
         <v>608</v>
       </c>
-      <c r="C106" s="317"/>
+      <c r="C106" s="319"/>
       <c r="D106" s="244">
         <v>350</v>
       </c>
@@ -27108,10 +27125,10 @@
       <c r="A107" s="260">
         <v>52</v>
       </c>
-      <c r="B107" s="316" t="s">
+      <c r="B107" s="318" t="s">
         <v>609</v>
       </c>
-      <c r="C107" s="317"/>
+      <c r="C107" s="319"/>
       <c r="D107" s="244">
         <v>0</v>
       </c>
@@ -27206,10 +27223,10 @@
       <c r="A109" s="23">
         <v>53</v>
       </c>
-      <c r="B109" s="320" t="s">
+      <c r="B109" s="316" t="s">
         <v>610</v>
       </c>
-      <c r="C109" s="321"/>
+      <c r="C109" s="317"/>
       <c r="D109" s="244">
         <v>2441</v>
       </c>
@@ -27259,10 +27276,10 @@
       <c r="A110" s="23">
         <v>54</v>
       </c>
-      <c r="B110" s="320" t="s">
+      <c r="B110" s="316" t="s">
         <v>611</v>
       </c>
-      <c r="C110" s="321"/>
+      <c r="C110" s="317"/>
       <c r="D110" s="244">
         <v>39</v>
       </c>
@@ -27311,10 +27328,10 @@
       <c r="A111" s="23">
         <v>55</v>
       </c>
-      <c r="B111" s="320" t="s">
+      <c r="B111" s="316" t="s">
         <v>612</v>
       </c>
-      <c r="C111" s="321"/>
+      <c r="C111" s="317"/>
       <c r="D111" s="244">
         <v>20</v>
       </c>
@@ -27365,10 +27382,10 @@
       <c r="A112" s="23">
         <v>56</v>
       </c>
-      <c r="B112" s="320" t="s">
+      <c r="B112" s="316" t="s">
         <v>613</v>
       </c>
-      <c r="C112" s="321"/>
+      <c r="C112" s="317"/>
       <c r="D112" s="244">
         <v>331</v>
       </c>
@@ -27417,10 +27434,10 @@
       <c r="A113" s="23">
         <v>57</v>
       </c>
-      <c r="B113" s="320" t="s">
+      <c r="B113" s="316" t="s">
         <v>614</v>
       </c>
-      <c r="C113" s="321"/>
+      <c r="C113" s="317"/>
       <c r="D113" s="244">
         <v>227</v>
       </c>
@@ -27468,10 +27485,10 @@
       <c r="A114" s="23">
         <v>58</v>
       </c>
-      <c r="B114" s="320" t="s">
+      <c r="B114" s="316" t="s">
         <v>615</v>
       </c>
-      <c r="C114" s="321"/>
+      <c r="C114" s="317"/>
       <c r="D114" s="244">
         <v>322</v>
       </c>
@@ -27522,10 +27539,10 @@
       <c r="A115" s="23">
         <v>59</v>
       </c>
-      <c r="B115" s="320" t="s">
+      <c r="B115" s="316" t="s">
         <v>616</v>
       </c>
-      <c r="C115" s="321"/>
+      <c r="C115" s="317"/>
       <c r="D115" s="244">
         <v>110</v>
       </c>
@@ -27576,10 +27593,10 @@
       <c r="A116" s="23">
         <v>60</v>
       </c>
-      <c r="B116" s="320" t="s">
+      <c r="B116" s="316" t="s">
         <v>617</v>
       </c>
-      <c r="C116" s="321"/>
+      <c r="C116" s="317"/>
       <c r="D116" s="244">
         <v>993</v>
       </c>
@@ -27630,10 +27647,10 @@
       <c r="A117" s="23">
         <v>61</v>
       </c>
-      <c r="B117" s="320" t="s">
+      <c r="B117" s="316" t="s">
         <v>618</v>
       </c>
-      <c r="C117" s="321"/>
+      <c r="C117" s="317"/>
       <c r="D117" s="244">
         <v>99</v>
       </c>
@@ -27684,10 +27701,10 @@
       <c r="A118" s="23">
         <v>62</v>
       </c>
-      <c r="B118" s="320" t="s">
+      <c r="B118" s="316" t="s">
         <v>619</v>
       </c>
-      <c r="C118" s="321"/>
+      <c r="C118" s="317"/>
       <c r="D118" s="244">
         <v>0</v>
       </c>
@@ -27738,10 +27755,10 @@
       <c r="A119" s="23">
         <v>63</v>
       </c>
-      <c r="B119" s="320" t="s">
+      <c r="B119" s="316" t="s">
         <v>620</v>
       </c>
-      <c r="C119" s="321"/>
+      <c r="C119" s="317"/>
       <c r="D119" s="244">
         <v>6</v>
       </c>
@@ -27792,10 +27809,10 @@
       <c r="A120" s="23">
         <v>64</v>
       </c>
-      <c r="B120" s="320" t="s">
+      <c r="B120" s="316" t="s">
         <v>621</v>
       </c>
-      <c r="C120" s="321"/>
+      <c r="C120" s="317"/>
       <c r="D120" s="244">
         <v>216</v>
       </c>
@@ -27846,10 +27863,10 @@
       <c r="A121" s="23">
         <v>65</v>
       </c>
-      <c r="B121" s="320" t="s">
+      <c r="B121" s="316" t="s">
         <v>622</v>
       </c>
-      <c r="C121" s="321"/>
+      <c r="C121" s="317"/>
       <c r="D121" s="244">
         <v>3013</v>
       </c>
@@ -27900,10 +27917,10 @@
       <c r="A122" s="23">
         <v>66</v>
       </c>
-      <c r="B122" s="320" t="s">
+      <c r="B122" s="316" t="s">
         <v>624</v>
       </c>
-      <c r="C122" s="321"/>
+      <c r="C122" s="317"/>
       <c r="D122" s="244">
         <v>59</v>
       </c>
@@ -27954,10 +27971,10 @@
       <c r="A123" s="23">
         <v>67</v>
       </c>
-      <c r="B123" s="320" t="s">
+      <c r="B123" s="316" t="s">
         <v>625</v>
       </c>
-      <c r="C123" s="321"/>
+      <c r="C123" s="317"/>
       <c r="D123" s="244">
         <v>189</v>
       </c>
@@ -28008,10 +28025,10 @@
       <c r="A124" s="23">
         <v>68</v>
       </c>
-      <c r="B124" s="320" t="s">
+      <c r="B124" s="316" t="s">
         <v>701</v>
       </c>
-      <c r="C124" s="321"/>
+      <c r="C124" s="317"/>
       <c r="D124" s="244">
         <v>174</v>
       </c>
@@ -28059,10 +28076,10 @@
       <c r="A125" s="23">
         <v>69</v>
       </c>
-      <c r="B125" s="320" t="s">
+      <c r="B125" s="316" t="s">
         <v>702</v>
       </c>
-      <c r="C125" s="321"/>
+      <c r="C125" s="317"/>
       <c r="D125" s="244">
         <v>137</v>
       </c>
@@ -28113,10 +28130,10 @@
       <c r="A126" s="23">
         <v>70</v>
       </c>
-      <c r="B126" s="320" t="s">
+      <c r="B126" s="316" t="s">
         <v>703</v>
       </c>
-      <c r="C126" s="321"/>
+      <c r="C126" s="317"/>
       <c r="D126" s="244">
         <v>2</v>
       </c>
@@ -28167,10 +28184,10 @@
       <c r="A127" s="23">
         <v>71</v>
       </c>
-      <c r="B127" s="320" t="s">
+      <c r="B127" s="316" t="s">
         <v>704</v>
       </c>
-      <c r="C127" s="321"/>
+      <c r="C127" s="317"/>
       <c r="D127" s="244">
         <v>341</v>
       </c>
@@ -28221,10 +28238,10 @@
       <c r="A128" s="23">
         <v>72</v>
       </c>
-      <c r="B128" s="320" t="s">
+      <c r="B128" s="316" t="s">
         <v>705</v>
       </c>
-      <c r="C128" s="321"/>
+      <c r="C128" s="317"/>
       <c r="D128" s="244">
         <v>20</v>
       </c>
@@ -28275,10 +28292,10 @@
       <c r="A129" s="23">
         <v>73</v>
       </c>
-      <c r="B129" s="320" t="s">
+      <c r="B129" s="316" t="s">
         <v>706</v>
       </c>
-      <c r="C129" s="321"/>
+      <c r="C129" s="317"/>
       <c r="D129" s="244">
         <v>621</v>
       </c>
@@ -28328,10 +28345,10 @@
       <c r="A130" s="23">
         <v>74</v>
       </c>
-      <c r="B130" s="320" t="s">
+      <c r="B130" s="316" t="s">
         <v>708</v>
       </c>
-      <c r="C130" s="321"/>
+      <c r="C130" s="317"/>
       <c r="D130" s="244">
         <v>1156</v>
       </c>
@@ -28382,10 +28399,10 @@
       <c r="A131" s="23">
         <v>75</v>
       </c>
-      <c r="B131" s="320" t="s">
+      <c r="B131" s="316" t="s">
         <v>709</v>
       </c>
-      <c r="C131" s="321"/>
+      <c r="C131" s="317"/>
       <c r="D131" s="244">
         <v>1826</v>
       </c>
@@ -28436,10 +28453,10 @@
       <c r="A132" s="23">
         <v>76</v>
       </c>
-      <c r="B132" s="320" t="s">
+      <c r="B132" s="316" t="s">
         <v>710</v>
       </c>
-      <c r="C132" s="321"/>
+      <c r="C132" s="317"/>
       <c r="D132" s="244">
         <v>0</v>
       </c>
@@ -28490,10 +28507,10 @@
       <c r="A133" s="23">
         <v>77</v>
       </c>
-      <c r="B133" s="320" t="s">
+      <c r="B133" s="316" t="s">
         <v>711</v>
       </c>
-      <c r="C133" s="321"/>
+      <c r="C133" s="317"/>
       <c r="D133" s="244">
         <v>30</v>
       </c>
@@ -28544,10 +28561,10 @@
       <c r="A134" s="23">
         <v>78</v>
       </c>
-      <c r="B134" s="320" t="s">
+      <c r="B134" s="316" t="s">
         <v>712</v>
       </c>
-      <c r="C134" s="321"/>
+      <c r="C134" s="317"/>
       <c r="D134" s="244">
         <v>16</v>
       </c>
@@ -28598,10 +28615,10 @@
       <c r="A135" s="23">
         <v>79</v>
       </c>
-      <c r="B135" s="320" t="s">
+      <c r="B135" s="316" t="s">
         <v>713</v>
       </c>
-      <c r="C135" s="321"/>
+      <c r="C135" s="317"/>
       <c r="D135" s="244">
         <v>4</v>
       </c>
@@ -28652,10 +28669,10 @@
       <c r="A136" s="23">
         <v>80</v>
       </c>
-      <c r="B136" s="320" t="s">
+      <c r="B136" s="316" t="s">
         <v>714</v>
       </c>
-      <c r="C136" s="321"/>
+      <c r="C136" s="317"/>
       <c r="D136" s="244">
         <v>176</v>
       </c>
@@ -28706,10 +28723,10 @@
       <c r="A137" s="23">
         <v>81</v>
       </c>
-      <c r="B137" s="320" t="s">
+      <c r="B137" s="316" t="s">
         <v>715</v>
       </c>
-      <c r="C137" s="321"/>
+      <c r="C137" s="317"/>
       <c r="D137" s="244">
         <v>246</v>
       </c>
@@ -28760,10 +28777,10 @@
       <c r="A138" s="23">
         <v>82</v>
       </c>
-      <c r="B138" s="320" t="s">
+      <c r="B138" s="316" t="s">
         <v>716</v>
       </c>
-      <c r="C138" s="321"/>
+      <c r="C138" s="317"/>
       <c r="D138" s="244">
         <v>0</v>
       </c>
@@ -28814,10 +28831,10 @@
       <c r="A139" s="23">
         <v>83</v>
       </c>
-      <c r="B139" s="320" t="s">
+      <c r="B139" s="316" t="s">
         <v>717</v>
       </c>
-      <c r="C139" s="321"/>
+      <c r="C139" s="317"/>
       <c r="D139" s="244">
         <v>0</v>
       </c>
@@ -28868,10 +28885,10 @@
       <c r="A140" s="23">
         <v>84</v>
       </c>
-      <c r="B140" s="320" t="s">
+      <c r="B140" s="316" t="s">
         <v>718</v>
       </c>
-      <c r="C140" s="321"/>
+      <c r="C140" s="317"/>
       <c r="D140" s="244">
         <v>14</v>
       </c>
@@ -28922,10 +28939,10 @@
       <c r="A141" s="23">
         <v>85</v>
       </c>
-      <c r="B141" s="320" t="s">
+      <c r="B141" s="316" t="s">
         <v>719</v>
       </c>
-      <c r="C141" s="321"/>
+      <c r="C141" s="317"/>
       <c r="D141" s="244">
         <v>47</v>
       </c>
@@ -28976,10 +28993,10 @@
       <c r="A142" s="23">
         <v>86</v>
       </c>
-      <c r="B142" s="320" t="s">
+      <c r="B142" s="316" t="s">
         <v>720</v>
       </c>
-      <c r="C142" s="321"/>
+      <c r="C142" s="317"/>
       <c r="D142" s="244">
         <v>0</v>
       </c>
@@ -29030,10 +29047,10 @@
       <c r="A143" s="23">
         <v>87</v>
       </c>
-      <c r="B143" s="320" t="s">
+      <c r="B143" s="316" t="s">
         <v>721</v>
       </c>
-      <c r="C143" s="321"/>
+      <c r="C143" s="317"/>
       <c r="D143" s="244">
         <v>55</v>
       </c>
@@ -29084,10 +29101,10 @@
       <c r="A144" s="23">
         <v>88</v>
       </c>
-      <c r="B144" s="320" t="s">
+      <c r="B144" s="316" t="s">
         <v>722</v>
       </c>
-      <c r="C144" s="321"/>
+      <c r="C144" s="317"/>
       <c r="D144" s="244">
         <v>7</v>
       </c>
@@ -29138,10 +29155,10 @@
       <c r="A145" s="23">
         <v>89</v>
       </c>
-      <c r="B145" s="320" t="s">
+      <c r="B145" s="316" t="s">
         <v>723</v>
       </c>
-      <c r="C145" s="321"/>
+      <c r="C145" s="317"/>
       <c r="D145" s="244">
         <v>80</v>
       </c>
@@ -29189,10 +29206,10 @@
       <c r="A146" s="23">
         <v>90</v>
       </c>
-      <c r="B146" s="320" t="s">
+      <c r="B146" s="316" t="s">
         <v>725</v>
       </c>
-      <c r="C146" s="321"/>
+      <c r="C146" s="317"/>
       <c r="D146" s="244">
         <v>0</v>
       </c>
@@ -29241,10 +29258,10 @@
       <c r="A147" s="23">
         <v>91</v>
       </c>
-      <c r="B147" s="320" t="s">
+      <c r="B147" s="316" t="s">
         <v>726</v>
       </c>
-      <c r="C147" s="321"/>
+      <c r="C147" s="317"/>
       <c r="D147" s="244">
         <v>0</v>
       </c>
@@ -29295,10 +29312,10 @@
       <c r="A148" s="23">
         <v>92</v>
       </c>
-      <c r="B148" s="320" t="s">
+      <c r="B148" s="316" t="s">
         <v>727</v>
       </c>
-      <c r="C148" s="321"/>
+      <c r="C148" s="317"/>
       <c r="D148" s="244">
         <v>0</v>
       </c>
@@ -29349,10 +29366,10 @@
       <c r="A149" s="23">
         <v>93</v>
       </c>
-      <c r="B149" s="320" t="s">
+      <c r="B149" s="316" t="s">
         <v>728</v>
       </c>
-      <c r="C149" s="321"/>
+      <c r="C149" s="317"/>
       <c r="D149" s="244">
         <v>0</v>
       </c>
@@ -29403,10 +29420,10 @@
       <c r="A150" s="23">
         <v>94</v>
       </c>
-      <c r="B150" s="320" t="s">
+      <c r="B150" s="316" t="s">
         <v>729</v>
       </c>
-      <c r="C150" s="321"/>
+      <c r="C150" s="317"/>
       <c r="D150" s="244">
         <v>0</v>
       </c>
@@ -29457,10 +29474,10 @@
       <c r="A151" s="23">
         <v>95</v>
       </c>
-      <c r="B151" s="320" t="s">
+      <c r="B151" s="316" t="s">
         <v>730</v>
       </c>
-      <c r="C151" s="321"/>
+      <c r="C151" s="317"/>
       <c r="D151" s="244">
         <v>0</v>
       </c>
@@ -29511,10 +29528,10 @@
       <c r="A152" s="23">
         <v>96</v>
       </c>
-      <c r="B152" s="320" t="s">
+      <c r="B152" s="316" t="s">
         <v>731</v>
       </c>
-      <c r="C152" s="321"/>
+      <c r="C152" s="317"/>
       <c r="D152" s="244">
         <v>60</v>
       </c>
@@ -29565,10 +29582,10 @@
       <c r="A153" s="23">
         <v>97</v>
       </c>
-      <c r="B153" s="320" t="s">
+      <c r="B153" s="316" t="s">
         <v>732</v>
       </c>
-      <c r="C153" s="321"/>
+      <c r="C153" s="317"/>
       <c r="D153" s="244">
         <v>0</v>
       </c>
@@ -29619,10 +29636,10 @@
       <c r="A154" s="23">
         <v>98</v>
       </c>
-      <c r="B154" s="320" t="s">
+      <c r="B154" s="316" t="s">
         <v>733</v>
       </c>
-      <c r="C154" s="321"/>
+      <c r="C154" s="317"/>
       <c r="D154" s="244"/>
       <c r="E154" s="244">
         <v>1789</v>
@@ -29671,10 +29688,10 @@
       <c r="A155" s="23">
         <v>99</v>
       </c>
-      <c r="B155" s="320" t="s">
+      <c r="B155" s="316" t="s">
         <v>735</v>
       </c>
-      <c r="C155" s="321"/>
+      <c r="C155" s="317"/>
       <c r="D155" s="244"/>
       <c r="E155" s="244">
         <v>64</v>
@@ -29719,10 +29736,10 @@
       <c r="A156" s="23">
         <v>100</v>
       </c>
-      <c r="B156" s="320" t="s">
+      <c r="B156" s="316" t="s">
         <v>736</v>
       </c>
-      <c r="C156" s="321"/>
+      <c r="C156" s="317"/>
       <c r="D156" s="244"/>
       <c r="E156" s="244">
         <v>763</v>
@@ -29771,10 +29788,10 @@
       <c r="A157" s="23">
         <v>101</v>
       </c>
-      <c r="B157" s="320" t="s">
+      <c r="B157" s="316" t="s">
         <v>738</v>
       </c>
-      <c r="C157" s="321"/>
+      <c r="C157" s="317"/>
       <c r="D157" s="244">
         <v>0</v>
       </c>
@@ -29825,10 +29842,10 @@
       <c r="A158" s="23">
         <v>102</v>
       </c>
-      <c r="B158" s="320" t="s">
+      <c r="B158" s="316" t="s">
         <v>739</v>
       </c>
-      <c r="C158" s="321"/>
+      <c r="C158" s="317"/>
       <c r="D158" s="244">
         <v>0</v>
       </c>
@@ -29879,10 +29896,10 @@
       <c r="A159" s="23">
         <v>103</v>
       </c>
-      <c r="B159" s="320" t="s">
+      <c r="B159" s="316" t="s">
         <v>740</v>
       </c>
-      <c r="C159" s="321"/>
+      <c r="C159" s="317"/>
       <c r="D159" s="244">
         <v>0</v>
       </c>
@@ -29933,10 +29950,10 @@
       <c r="A160" s="23">
         <v>104</v>
       </c>
-      <c r="B160" s="320" t="s">
+      <c r="B160" s="316" t="s">
         <v>741</v>
       </c>
-      <c r="C160" s="321"/>
+      <c r="C160" s="317"/>
       <c r="D160" s="244">
         <v>408</v>
       </c>
@@ -29987,10 +30004,10 @@
       <c r="A161" s="23">
         <v>105</v>
       </c>
-      <c r="B161" s="320" t="s">
+      <c r="B161" s="316" t="s">
         <v>742</v>
       </c>
-      <c r="C161" s="321"/>
+      <c r="C161" s="317"/>
       <c r="D161" s="244">
         <v>0</v>
       </c>
@@ -30041,10 +30058,10 @@
       <c r="A162" s="23">
         <v>106</v>
       </c>
-      <c r="B162" s="320" t="s">
+      <c r="B162" s="316" t="s">
         <v>743</v>
       </c>
-      <c r="C162" s="321"/>
+      <c r="C162" s="317"/>
       <c r="D162" s="244">
         <v>0</v>
       </c>
@@ -30095,10 +30112,10 @@
       <c r="A163" s="23">
         <v>107</v>
       </c>
-      <c r="B163" s="320" t="s">
+      <c r="B163" s="316" t="s">
         <v>744</v>
       </c>
-      <c r="C163" s="321"/>
+      <c r="C163" s="317"/>
       <c r="D163" s="244">
         <v>0</v>
       </c>
@@ -30149,10 +30166,10 @@
       <c r="A164" s="23">
         <v>108</v>
       </c>
-      <c r="B164" s="320" t="s">
+      <c r="B164" s="316" t="s">
         <v>745</v>
       </c>
-      <c r="C164" s="321"/>
+      <c r="C164" s="317"/>
       <c r="D164" s="244">
         <v>0</v>
       </c>
@@ -30203,10 +30220,10 @@
       <c r="A165" s="23">
         <v>109</v>
       </c>
-      <c r="B165" s="320" t="s">
+      <c r="B165" s="316" t="s">
         <v>746</v>
       </c>
-      <c r="C165" s="321"/>
+      <c r="C165" s="317"/>
       <c r="D165" s="244">
         <v>0</v>
       </c>
@@ -30257,10 +30274,10 @@
       <c r="A166" s="23">
         <v>110</v>
       </c>
-      <c r="B166" s="320" t="s">
+      <c r="B166" s="316" t="s">
         <v>747</v>
       </c>
-      <c r="C166" s="321"/>
+      <c r="C166" s="317"/>
       <c r="D166" s="244">
         <v>0</v>
       </c>
@@ -30311,10 +30328,10 @@
       <c r="A167" s="23">
         <v>111</v>
       </c>
-      <c r="B167" s="320" t="s">
+      <c r="B167" s="316" t="s">
         <v>748</v>
       </c>
-      <c r="C167" s="321"/>
+      <c r="C167" s="317"/>
       <c r="D167" s="244">
         <v>3</v>
       </c>
@@ -30365,10 +30382,10 @@
       <c r="A168" s="23">
         <v>112</v>
       </c>
-      <c r="B168" s="320" t="s">
+      <c r="B168" s="316" t="s">
         <v>750</v>
       </c>
-      <c r="C168" s="321"/>
+      <c r="C168" s="317"/>
       <c r="D168" s="244">
         <v>0</v>
       </c>
@@ -30419,10 +30436,10 @@
       <c r="A169" s="270">
         <v>113</v>
       </c>
-      <c r="B169" s="320" t="s">
+      <c r="B169" s="316" t="s">
         <v>752</v>
       </c>
-      <c r="C169" s="321"/>
+      <c r="C169" s="317"/>
       <c r="D169" s="244">
         <v>0</v>
       </c>
@@ -30473,10 +30490,10 @@
       <c r="A170" s="270">
         <v>114</v>
       </c>
-      <c r="B170" s="320" t="s">
+      <c r="B170" s="316" t="s">
         <v>753</v>
       </c>
-      <c r="C170" s="321"/>
+      <c r="C170" s="317"/>
       <c r="D170" s="244">
         <v>0</v>
       </c>
@@ -30525,6 +30542,108 @@
     </row>
   </sheetData>
   <mergeCells count="115">
+    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A6:A11"/>
+    <mergeCell ref="A12:A15"/>
+    <mergeCell ref="A16:A21"/>
+    <mergeCell ref="A22:A26"/>
+    <mergeCell ref="A27:A29"/>
+    <mergeCell ref="A57:A58"/>
+    <mergeCell ref="A59:A61"/>
+    <mergeCell ref="A62:A64"/>
+    <mergeCell ref="A65:A67"/>
+    <mergeCell ref="B69:C69"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="A30:A35"/>
+    <mergeCell ref="A36:A40"/>
+    <mergeCell ref="A41:A43"/>
+    <mergeCell ref="A44:A48"/>
+    <mergeCell ref="A49:A53"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B78:C78"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="B93:C93"/>
+    <mergeCell ref="B94:C94"/>
+    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="B96:C96"/>
+    <mergeCell ref="B84:C84"/>
+    <mergeCell ref="B85:C85"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B87:C87"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B103:C103"/>
+    <mergeCell ref="B104:C104"/>
+    <mergeCell ref="B105:C105"/>
+    <mergeCell ref="B106:C106"/>
+    <mergeCell ref="B107:C107"/>
+    <mergeCell ref="B109:C109"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B98:C98"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="B100:C100"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="B116:C116"/>
+    <mergeCell ref="B117:C117"/>
+    <mergeCell ref="B118:C118"/>
+    <mergeCell ref="B119:C119"/>
+    <mergeCell ref="B120:C120"/>
+    <mergeCell ref="B121:C121"/>
+    <mergeCell ref="B110:C110"/>
+    <mergeCell ref="B111:C111"/>
+    <mergeCell ref="B112:C112"/>
+    <mergeCell ref="B113:C113"/>
+    <mergeCell ref="B114:C114"/>
+    <mergeCell ref="B115:C115"/>
+    <mergeCell ref="B128:C128"/>
+    <mergeCell ref="B129:C129"/>
+    <mergeCell ref="B130:C130"/>
+    <mergeCell ref="B131:C131"/>
+    <mergeCell ref="B132:C132"/>
+    <mergeCell ref="B133:C133"/>
+    <mergeCell ref="B122:C122"/>
+    <mergeCell ref="B123:C123"/>
+    <mergeCell ref="B124:C124"/>
+    <mergeCell ref="B125:C125"/>
+    <mergeCell ref="B126:C126"/>
+    <mergeCell ref="B127:C127"/>
+    <mergeCell ref="B140:C140"/>
+    <mergeCell ref="B141:C141"/>
+    <mergeCell ref="B142:C142"/>
+    <mergeCell ref="B143:C143"/>
+    <mergeCell ref="B144:C144"/>
+    <mergeCell ref="B145:C145"/>
+    <mergeCell ref="B134:C134"/>
+    <mergeCell ref="B135:C135"/>
+    <mergeCell ref="B136:C136"/>
+    <mergeCell ref="B137:C137"/>
+    <mergeCell ref="B138:C138"/>
+    <mergeCell ref="B139:C139"/>
+    <mergeCell ref="B152:C152"/>
+    <mergeCell ref="B153:C153"/>
+    <mergeCell ref="B154:C154"/>
+    <mergeCell ref="B155:C155"/>
+    <mergeCell ref="B156:C156"/>
+    <mergeCell ref="B157:C157"/>
+    <mergeCell ref="B146:C146"/>
+    <mergeCell ref="B147:C147"/>
+    <mergeCell ref="B148:C148"/>
+    <mergeCell ref="B149:C149"/>
+    <mergeCell ref="B150:C150"/>
+    <mergeCell ref="B151:C151"/>
     <mergeCell ref="B170:C170"/>
     <mergeCell ref="B164:C164"/>
     <mergeCell ref="B165:C165"/>
@@ -30538,108 +30657,6 @@
     <mergeCell ref="B161:C161"/>
     <mergeCell ref="B162:C162"/>
     <mergeCell ref="B163:C163"/>
-    <mergeCell ref="B152:C152"/>
-    <mergeCell ref="B153:C153"/>
-    <mergeCell ref="B154:C154"/>
-    <mergeCell ref="B155:C155"/>
-    <mergeCell ref="B156:C156"/>
-    <mergeCell ref="B157:C157"/>
-    <mergeCell ref="B146:C146"/>
-    <mergeCell ref="B147:C147"/>
-    <mergeCell ref="B148:C148"/>
-    <mergeCell ref="B149:C149"/>
-    <mergeCell ref="B150:C150"/>
-    <mergeCell ref="B151:C151"/>
-    <mergeCell ref="B140:C140"/>
-    <mergeCell ref="B141:C141"/>
-    <mergeCell ref="B142:C142"/>
-    <mergeCell ref="B143:C143"/>
-    <mergeCell ref="B144:C144"/>
-    <mergeCell ref="B145:C145"/>
-    <mergeCell ref="B134:C134"/>
-    <mergeCell ref="B135:C135"/>
-    <mergeCell ref="B136:C136"/>
-    <mergeCell ref="B137:C137"/>
-    <mergeCell ref="B138:C138"/>
-    <mergeCell ref="B139:C139"/>
-    <mergeCell ref="B128:C128"/>
-    <mergeCell ref="B129:C129"/>
-    <mergeCell ref="B130:C130"/>
-    <mergeCell ref="B131:C131"/>
-    <mergeCell ref="B132:C132"/>
-    <mergeCell ref="B133:C133"/>
-    <mergeCell ref="B122:C122"/>
-    <mergeCell ref="B123:C123"/>
-    <mergeCell ref="B124:C124"/>
-    <mergeCell ref="B125:C125"/>
-    <mergeCell ref="B126:C126"/>
-    <mergeCell ref="B127:C127"/>
-    <mergeCell ref="B116:C116"/>
-    <mergeCell ref="B117:C117"/>
-    <mergeCell ref="B118:C118"/>
-    <mergeCell ref="B119:C119"/>
-    <mergeCell ref="B120:C120"/>
-    <mergeCell ref="B121:C121"/>
-    <mergeCell ref="B110:C110"/>
-    <mergeCell ref="B111:C111"/>
-    <mergeCell ref="B112:C112"/>
-    <mergeCell ref="B113:C113"/>
-    <mergeCell ref="B114:C114"/>
-    <mergeCell ref="B115:C115"/>
-    <mergeCell ref="B103:C103"/>
-    <mergeCell ref="B104:C104"/>
-    <mergeCell ref="B105:C105"/>
-    <mergeCell ref="B106:C106"/>
-    <mergeCell ref="B107:C107"/>
-    <mergeCell ref="B109:C109"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B98:C98"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="B100:C100"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="B102:C102"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B95:C95"/>
-    <mergeCell ref="B96:C96"/>
-    <mergeCell ref="B84:C84"/>
-    <mergeCell ref="B85:C85"/>
-    <mergeCell ref="B86:C86"/>
-    <mergeCell ref="B87:C87"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B90:C90"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="A65:A67"/>
-    <mergeCell ref="B69:C69"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="A30:A35"/>
-    <mergeCell ref="A36:A40"/>
-    <mergeCell ref="A41:A43"/>
-    <mergeCell ref="A44:A48"/>
-    <mergeCell ref="A49:A53"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="A2:P2"/>
-    <mergeCell ref="A6:A11"/>
-    <mergeCell ref="A12:A15"/>
-    <mergeCell ref="A16:A21"/>
-    <mergeCell ref="A22:A26"/>
-    <mergeCell ref="A27:A29"/>
-    <mergeCell ref="A57:A58"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="A62:A64"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:K170" xr:uid="{CC92B26A-0E54-4215-9F91-552807E30F43}">
@@ -30666,52 +30683,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="322" t="s">
+      <c r="A1" s="326" t="s">
         <v>128</v>
       </c>
-      <c r="B1" s="322"/>
-      <c r="C1" s="322"/>
-      <c r="D1" s="322"/>
-      <c r="E1" s="322"/>
-      <c r="F1" s="322"/>
-      <c r="G1" s="322"/>
-      <c r="H1" s="322"/>
-      <c r="I1" s="322"/>
-      <c r="J1" s="322"/>
-      <c r="K1" s="322"/>
-      <c r="L1" s="322"/>
+      <c r="B1" s="326"/>
+      <c r="C1" s="326"/>
+      <c r="D1" s="326"/>
+      <c r="E1" s="326"/>
+      <c r="F1" s="326"/>
+      <c r="G1" s="326"/>
+      <c r="H1" s="326"/>
+      <c r="I1" s="326"/>
+      <c r="J1" s="326"/>
+      <c r="K1" s="326"/>
+      <c r="L1" s="326"/>
     </row>
     <row r="2" spans="1:12" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="323" t="s">
+      <c r="A2" s="327" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="324" t="s">
+      <c r="B2" s="328" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="323" t="s">
+      <c r="C2" s="327" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="323"/>
-      <c r="E2" s="323" t="s">
+      <c r="D2" s="327"/>
+      <c r="E2" s="327" t="s">
         <v>130</v>
       </c>
-      <c r="F2" s="323"/>
-      <c r="G2" s="323"/>
-      <c r="H2" s="323"/>
-      <c r="I2" s="323"/>
-      <c r="J2" s="323" t="s">
+      <c r="F2" s="327"/>
+      <c r="G2" s="327"/>
+      <c r="H2" s="327"/>
+      <c r="I2" s="327"/>
+      <c r="J2" s="327" t="s">
         <v>130</v>
       </c>
-      <c r="K2" s="325" t="s">
+      <c r="K2" s="329" t="s">
         <v>136</v>
       </c>
-      <c r="L2" s="323" t="s">
+      <c r="L2" s="327" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="323"/>
-      <c r="B3" s="324"/>
+      <c r="A3" s="327"/>
+      <c r="B3" s="328"/>
       <c r="C3" s="83" t="s">
         <v>131</v>
       </c>
@@ -30733,9 +30750,9 @@
       <c r="I3" s="83" t="s">
         <v>127</v>
       </c>
-      <c r="J3" s="323"/>
-      <c r="K3" s="326"/>
-      <c r="L3" s="323"/>
+      <c r="J3" s="327"/>
+      <c r="K3" s="330"/>
+      <c r="L3" s="327"/>
     </row>
     <row r="4" spans="1:12" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="85">

</xml_diff>